<commit_message>
phase3(#5,#12): AP เครดิตเทอม+DPO+AP aging, คอลัมน์ fixed/variable, ขยาย expenses schema
</commit_message>
<xml_diff>
--- a/WAYTHAI-FORYOU_Template.xlsx
+++ b/WAYTHAI-FORYOU_Template.xlsx
@@ -285,6 +285,13 @@
         <t>ค่าสีและวัสดุทุกชนิด บันทึกที่ชีตนี้
 เลือก category = paint / wood / hardware / labor
 (ไม่มีชีต material แยกแล้ว)</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>ซื้อเชื่อ: ใส่จำนวนวันเครดิต (30/45/60)
+จ่ายเงินสดทันที: ใส่ 0
+ระบบใช้คำนวณ AP/เจ้าหนี้ + DPO</t>
       </text>
     </comment>
   </commentList>
@@ -692,7 +699,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="13" t="inlineStr"/>
     </row>
@@ -3077,7 +3083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3085,6 +3091,8 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3113,6 +3121,16 @@
           <t>รายการ/หมายเหตุ (เช่น ร้านที่ซื้อ/แบรนด์สี)</t>
         </is>
       </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>เครดิตเทอม (วัน)  — เงินสดใส่ 0</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>ประเภท (คงที่/ผันแปร)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -3138,6 +3156,16 @@
       <c r="E2" s="7" t="inlineStr">
         <is>
           <t>note</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>credit_term</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>expense_kind</t>
         </is>
       </c>
     </row>
@@ -4128,13 +4156,19 @@
       <c r="B200" s="12" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="B3:B500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="วันที่ไม่ถูกต้อง" error="ต้องเป็นวันที่ ค.ศ (ปี 2020–2035) เช่น 15/06/2026 — ถ้าพิมพ์ พ.ศ (เช่น 2569) จะไม่ผ่าน" promptTitle="รูปแบบวันที่ (ค.ศ)" prompt="กรอก วว/ดด/ปปปป (ค.ศ) เช่น 15/06/2026  •  ห้ามใช้ พ.ศ" type="date" operator="between">
       <formula1>DATE(2020,1,1)</formula1>
       <formula2>DATE(2035,12,31)</formula2>
     </dataValidation>
     <dataValidation sqref="C3:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"paint,wood,hardware,labor,marketing,ads,rent,utility,overhead,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G3:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="ประเภทค่าใช้จ่าย" prompt="fixed = คงที่ (เช่า/เงินเดือน) | variable = ผันแปร (วัสดุ/ค่าสี)" type="list">
+      <formula1>"fixed,variable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F3:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="เครดิตเทอม (วัน)" prompt="ซื้อเชื่อกี่วัน เช่น 30/45/60 — ถ้าจ่ายเงินสดทันทีใส่ 0" type="whole" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>